<commit_message>
fix dashboard limit and sorting
</commit_message>
<xml_diff>
--- a/Corn.xlsx
+++ b/Corn.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://adm-my.sharepoint.com/personal/zeina_sherif_adm-medsofts_com/Documents/Documents/Commodity/Corn/Local/Model Daily/Dec-Jan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1272" documentId="8_{AFCAEB6C-147E-4472-A3AB-607E8F77BA32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F165DD4-68FC-430A-B567-5F02FA85D4D4}"/>
+  <xr:revisionPtr revIDLastSave="1048" documentId="8_{AFCAEB6C-147E-4472-A3AB-607E8F77BA32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDE80153-A8C4-496D-A044-C98BE0EC6C59}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{ECBE9064-6697-4608-8A07-17622AF5FF71}"/>
   </bookViews>
@@ -106,7 +106,7 @@
     <numFmt numFmtId="166" formatCode="[$-409]mmm\-yy;@"/>
     <numFmt numFmtId="167" formatCode="[$EGP]\ #,##0.00"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,15 +142,8 @@
       <family val="1"/>
       <scheme val="major"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Cambria"/>
-      <family val="1"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -178,18 +171,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -247,7 +228,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -262,9 +243,11 @@
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
@@ -272,18 +255,6 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -632,29 +603,27 @@
   <dimension ref="A1:S36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" customWidth="1"/>
+    <col min="5" max="5" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="11.81640625" customWidth="1"/>
+    <col min="9" max="9" width="16.08984375" customWidth="1"/>
+    <col min="10" max="10" width="11.81640625" customWidth="1"/>
+    <col min="11" max="11" width="15.26953125" customWidth="1"/>
+    <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
@@ -666,22 +635,22 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="13" t="s">
         <v>8</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -702,21 +671,21 @@
       <c r="P1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="18" t="s">
+      <c r="Q1" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="18" t="s">
+      <c r="R1" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="18" t="s">
+      <c r="S1" s="20" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A2" s="22">
+      <c r="A2" s="10">
         <v>45292</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="11">
         <v>380</v>
       </c>
       <c r="C2" s="2">
@@ -749,36 +718,30 @@
       <c r="K2" s="8">
         <v>16296.77</v>
       </c>
-      <c r="L2" s="14">
+      <c r="L2" s="16">
         <v>218.18</v>
       </c>
-      <c r="M2" s="23">
+      <c r="M2" s="16">
         <v>180.32</v>
       </c>
       <c r="N2" s="8">
         <v>16296.77</v>
       </c>
-      <c r="O2" s="14">
+      <c r="O2" s="16">
         <v>218.18</v>
       </c>
-      <c r="P2" s="23">
+      <c r="P2" s="16">
         <v>180.32</v>
       </c>
-      <c r="Q2" s="8">
-        <v>15216.13</v>
-      </c>
-      <c r="R2" s="19">
-        <v>172.01</v>
-      </c>
-      <c r="S2" s="24">
-        <v>107.53</v>
-      </c>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A3" s="22">
+      <c r="A3" s="10">
         <v>45323</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="11">
         <v>380</v>
       </c>
       <c r="C3" s="2">
@@ -812,36 +775,30 @@
       <c r="K3" s="8">
         <v>16544.830000000002</v>
       </c>
-      <c r="L3" s="14">
+      <c r="L3" s="16">
         <v>242.66</v>
       </c>
-      <c r="M3" s="23">
+      <c r="M3" s="16">
         <v>168.62</v>
       </c>
       <c r="N3" s="8">
         <v>16544.830000000002</v>
       </c>
-      <c r="O3" s="14">
+      <c r="O3" s="16">
         <v>242.66</v>
       </c>
-      <c r="P3" s="23">
+      <c r="P3" s="16">
         <v>180.32</v>
       </c>
-      <c r="Q3" s="8">
-        <v>15524.14</v>
-      </c>
-      <c r="R3" s="19">
-        <v>199.88</v>
-      </c>
-      <c r="S3" s="24">
-        <v>85.29</v>
-      </c>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A4" s="22">
+      <c r="A4" s="10">
         <v>45352</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="11">
         <v>380</v>
       </c>
       <c r="C4" s="2">
@@ -875,36 +832,30 @@
       <c r="K4" s="8">
         <v>12670.97</v>
       </c>
-      <c r="L4" s="14">
+      <c r="L4" s="16">
         <v>219.08</v>
       </c>
-      <c r="M4" s="23">
+      <c r="M4" s="16">
         <v>158.38999999999999</v>
       </c>
       <c r="N4" s="8">
         <v>12670.97</v>
       </c>
-      <c r="O4" s="14">
+      <c r="O4" s="16">
         <v>219.08</v>
       </c>
-      <c r="P4" s="23">
+      <c r="P4" s="16">
         <v>158.38999999999999</v>
       </c>
-      <c r="Q4" s="8">
-        <v>11254.84</v>
-      </c>
-      <c r="R4" s="19">
-        <v>143.55000000000001</v>
-      </c>
-      <c r="S4" s="24">
-        <v>90.19</v>
-      </c>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="21"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A5" s="22">
+      <c r="A5" s="10">
         <v>45383</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="11">
         <v>459</v>
       </c>
       <c r="C5" s="2">
@@ -938,36 +889,30 @@
       <c r="K5" s="8">
         <v>12430</v>
       </c>
-      <c r="L5" s="14">
+      <c r="L5" s="16">
         <v>199.27</v>
       </c>
-      <c r="M5" s="23">
+      <c r="M5" s="16">
         <v>150</v>
       </c>
       <c r="N5" s="8">
         <v>12430</v>
       </c>
-      <c r="O5" s="14">
+      <c r="O5" s="16">
         <v>199.27</v>
       </c>
-      <c r="P5" s="23">
+      <c r="P5" s="16">
         <v>150</v>
       </c>
-      <c r="Q5" s="8">
-        <v>11223.33</v>
-      </c>
-      <c r="R5" s="19">
-        <v>135.35</v>
-      </c>
-      <c r="S5" s="24">
-        <v>93.05</v>
-      </c>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="21"/>
+      <c r="S5" s="21"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A6" s="22">
+      <c r="A6" s="10">
         <v>45413</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="11">
         <v>459</v>
       </c>
       <c r="C6" s="2">
@@ -1001,36 +946,30 @@
       <c r="K6" s="8">
         <v>12048.39</v>
       </c>
-      <c r="L6" s="14">
+      <c r="L6" s="16">
         <v>159.97</v>
       </c>
-      <c r="M6" s="23">
+      <c r="M6" s="16">
         <v>150</v>
       </c>
       <c r="N6" s="8">
         <v>12048.39</v>
       </c>
-      <c r="O6" s="14">
+      <c r="O6" s="16">
         <v>159.97</v>
       </c>
-      <c r="P6" s="23">
+      <c r="P6" s="16">
         <v>150</v>
       </c>
-      <c r="Q6" s="8">
-        <v>10690.32</v>
-      </c>
-      <c r="R6" s="19">
-        <v>87.22</v>
-      </c>
-      <c r="S6" s="24">
-        <v>96.1</v>
-      </c>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A7" s="22">
+      <c r="A7" s="10">
         <v>45444</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="11">
         <v>459</v>
       </c>
       <c r="C7" s="2">
@@ -1064,36 +1003,30 @@
       <c r="K7" s="8">
         <v>11926.67</v>
       </c>
-      <c r="L7" s="14">
+      <c r="L7" s="16">
         <v>169.21</v>
       </c>
-      <c r="M7" s="23">
+      <c r="M7" s="16">
         <v>145</v>
       </c>
       <c r="N7" s="8">
         <v>11926.67</v>
       </c>
-      <c r="O7" s="14">
+      <c r="O7" s="16">
         <v>169.21</v>
       </c>
-      <c r="P7" s="23">
+      <c r="P7" s="16">
         <v>135</v>
       </c>
-      <c r="Q7" s="8">
-        <v>10880</v>
-      </c>
-      <c r="R7" s="19">
-        <v>113.69</v>
-      </c>
-      <c r="S7" s="24">
-        <v>130.66999999999999</v>
-      </c>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="S7" s="21"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A8" s="22">
+      <c r="A8" s="10">
         <v>45474</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="11">
         <v>459</v>
       </c>
       <c r="C8" s="2">
@@ -1127,36 +1060,30 @@
       <c r="K8" s="8">
         <v>11429.03</v>
       </c>
-      <c r="L8" s="14">
+      <c r="L8" s="16">
         <v>189.6</v>
       </c>
-      <c r="M8" s="23">
+      <c r="M8" s="16">
         <v>174.3</v>
       </c>
       <c r="N8" s="8">
         <v>11429.03</v>
       </c>
-      <c r="O8" s="14">
+      <c r="O8" s="16">
         <v>189.6</v>
       </c>
-      <c r="P8" s="23">
+      <c r="P8" s="16">
         <v>158.29</v>
       </c>
-      <c r="Q8" s="8">
-        <v>10696.77</v>
-      </c>
-      <c r="R8" s="19">
-        <v>151.16</v>
-      </c>
-      <c r="S8" s="24">
-        <v>150.21</v>
-      </c>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="S8" s="21"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A9" s="22">
+      <c r="A9" s="10">
         <v>45505</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="11">
         <v>459</v>
       </c>
       <c r="C9" s="2">
@@ -1190,36 +1117,30 @@
       <c r="K9" s="8">
         <v>11588.71</v>
       </c>
-      <c r="L9" s="15">
+      <c r="L9" s="17">
         <v>192.56</v>
       </c>
-      <c r="M9" s="23">
+      <c r="M9" s="16">
         <v>162.13</v>
       </c>
       <c r="N9" s="8">
         <v>11588.71</v>
       </c>
-      <c r="O9" s="14">
+      <c r="O9" s="16">
         <v>192.56</v>
       </c>
-      <c r="P9" s="23">
+      <c r="P9" s="16">
         <v>162.13</v>
       </c>
-      <c r="Q9" s="8">
-        <v>10958.06</v>
-      </c>
-      <c r="R9" s="19">
-        <v>159.88999999999999</v>
-      </c>
-      <c r="S9" s="24">
-        <v>182.6</v>
-      </c>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="21"/>
+      <c r="S9" s="21"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A10" s="22">
+      <c r="A10" s="10">
         <v>45536</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="11">
         <v>459</v>
       </c>
       <c r="C10" s="2">
@@ -1253,36 +1174,30 @@
       <c r="K10" s="8">
         <v>11693.33</v>
       </c>
-      <c r="L10" s="13">
+      <c r="L10" s="15">
         <v>177.71</v>
       </c>
-      <c r="M10" s="23">
+      <c r="M10" s="16">
         <v>178.9</v>
       </c>
       <c r="N10" s="8">
         <v>11693.33</v>
       </c>
-      <c r="O10" s="14">
+      <c r="O10" s="16">
         <v>177.71</v>
       </c>
-      <c r="P10" s="23">
+      <c r="P10" s="16">
         <v>173.9</v>
       </c>
-      <c r="Q10" s="8">
-        <v>11113.33</v>
-      </c>
-      <c r="R10" s="19">
-        <v>147.37</v>
-      </c>
-      <c r="S10" s="24">
-        <v>168.21</v>
-      </c>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="21"/>
+      <c r="S10" s="21"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A11" s="22">
+      <c r="A11" s="10">
         <v>45566</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="11">
         <v>500</v>
       </c>
       <c r="C11" s="2">
@@ -1316,36 +1231,30 @@
       <c r="K11" s="8">
         <v>12090.32</v>
       </c>
-      <c r="L11" s="13">
+      <c r="L11" s="15">
         <v>189.42</v>
       </c>
-      <c r="M11" s="23">
+      <c r="M11" s="16">
         <v>195.65</v>
       </c>
       <c r="N11" s="8">
         <v>12090.32</v>
       </c>
-      <c r="O11" s="14">
+      <c r="O11" s="16">
         <v>189.42</v>
       </c>
-      <c r="P11" s="23">
+      <c r="P11" s="16">
         <v>190.65</v>
       </c>
-      <c r="Q11" s="8">
-        <v>11658.06</v>
-      </c>
-      <c r="R11" s="19">
-        <v>166.83</v>
-      </c>
-      <c r="S11" s="24">
-        <v>195.7</v>
-      </c>
+      <c r="Q11" s="21"/>
+      <c r="R11" s="21"/>
+      <c r="S11" s="21"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A12" s="22">
+      <c r="A12" s="10">
         <v>45597</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="11">
         <v>515</v>
       </c>
       <c r="C12" s="2">
@@ -1379,36 +1288,30 @@
       <c r="K12" s="8">
         <v>12566.67</v>
       </c>
-      <c r="L12" s="13">
+      <c r="L12" s="15">
         <v>183.66</v>
       </c>
-      <c r="M12" s="23">
+      <c r="M12" s="16">
         <v>197.67</v>
       </c>
       <c r="N12" s="8">
         <v>12582.76</v>
       </c>
-      <c r="O12" s="14">
+      <c r="O12" s="16">
         <v>183.66</v>
       </c>
-      <c r="P12" s="23">
+      <c r="P12" s="16">
         <v>192.67</v>
       </c>
-      <c r="Q12" s="8">
-        <v>12226.67</v>
-      </c>
-      <c r="R12" s="19">
-        <v>166.21</v>
-      </c>
-      <c r="S12" s="24">
-        <v>157.96</v>
-      </c>
+      <c r="Q12" s="21"/>
+      <c r="R12" s="21"/>
+      <c r="S12" s="21"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A13" s="22">
+      <c r="A13" s="10">
         <v>45627</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="11">
         <v>515</v>
       </c>
       <c r="C13" s="2">
@@ -1432,7 +1335,7 @@
         <v>940000</v>
       </c>
       <c r="I13" s="6">
-        <f t="shared" ref="I13:I27" si="4">G13-H13</f>
+        <f t="shared" ref="I13:I26" si="4">G13-H13</f>
         <v>1118000</v>
       </c>
       <c r="J13" s="9">
@@ -1442,36 +1345,30 @@
       <c r="K13" s="8">
         <v>12872.58</v>
       </c>
-      <c r="L13" s="13">
+      <c r="L13" s="15">
         <v>175.53</v>
       </c>
-      <c r="M13" s="23">
+      <c r="M13" s="16">
         <v>174.45</v>
       </c>
       <c r="N13" s="8">
         <v>12872.58</v>
       </c>
-      <c r="O13" s="14">
+      <c r="O13" s="16">
         <v>175.53</v>
       </c>
-      <c r="P13" s="23">
+      <c r="P13" s="16">
         <v>169.74</v>
       </c>
-      <c r="Q13" s="8">
-        <v>12458.06</v>
-      </c>
-      <c r="R13" s="19">
-        <v>154.75</v>
-      </c>
-      <c r="S13" s="24">
-        <v>150.72</v>
-      </c>
+      <c r="Q13" s="21"/>
+      <c r="R13" s="21"/>
+      <c r="S13" s="21"/>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A14" s="22">
+      <c r="A14" s="10">
         <v>45658</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="11">
         <v>515</v>
       </c>
       <c r="C14" s="2">
@@ -1504,36 +1401,30 @@
       <c r="K14" s="8">
         <v>13335.48</v>
       </c>
-      <c r="L14" s="14">
+      <c r="L14" s="16">
         <v>170.96</v>
       </c>
-      <c r="M14" s="23">
+      <c r="M14" s="16">
         <v>176.58</v>
       </c>
       <c r="N14" s="8">
         <v>13335.48</v>
       </c>
-      <c r="O14" s="14">
+      <c r="O14" s="16">
         <v>170.96</v>
       </c>
-      <c r="P14" s="23">
+      <c r="P14" s="16">
         <v>175.55</v>
       </c>
-      <c r="Q14" s="8">
-        <v>12580.65</v>
-      </c>
-      <c r="R14" s="19">
-        <v>132.97</v>
-      </c>
-      <c r="S14" s="24">
-        <v>126.63</v>
-      </c>
+      <c r="Q14" s="21"/>
+      <c r="R14" s="21"/>
+      <c r="S14" s="21"/>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A15" s="22">
+      <c r="A15" s="10">
         <v>45689</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="11">
         <v>515</v>
       </c>
       <c r="C15" s="2">
@@ -1567,36 +1458,30 @@
       <c r="K15" s="8">
         <v>13435.71</v>
       </c>
-      <c r="L15" s="14">
+      <c r="L15" s="16">
         <v>160.66999999999999</v>
       </c>
-      <c r="M15" s="23">
+      <c r="M15" s="16">
         <v>182.14</v>
       </c>
       <c r="N15" s="8">
         <v>13435.71</v>
       </c>
-      <c r="O15" s="14">
+      <c r="O15" s="16">
         <v>160.66999999999999</v>
       </c>
-      <c r="P15" s="23">
+      <c r="P15" s="16">
         <v>180.71</v>
       </c>
-      <c r="Q15" s="8">
-        <v>12546.43</v>
-      </c>
-      <c r="R15" s="19">
-        <v>235.67</v>
-      </c>
-      <c r="S15" s="24">
-        <v>120.45</v>
-      </c>
+      <c r="Q15" s="21"/>
+      <c r="R15" s="21"/>
+      <c r="S15" s="21"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A16" s="22">
+      <c r="A16" s="10">
         <v>45717</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="11">
         <v>515</v>
       </c>
       <c r="C16" s="2">
@@ -1630,36 +1515,30 @@
       <c r="K16" s="8">
         <v>13117.74</v>
       </c>
-      <c r="L16" s="14">
+      <c r="L16" s="16">
         <v>170.75466969999999</v>
       </c>
-      <c r="M16" s="23">
+      <c r="M16" s="16">
         <v>186.32</v>
       </c>
       <c r="N16" s="8">
         <v>13117.74</v>
       </c>
-      <c r="O16" s="14">
+      <c r="O16" s="16">
         <v>170.75</v>
       </c>
-      <c r="P16" s="23">
+      <c r="P16" s="16">
         <v>186.32</v>
       </c>
-      <c r="Q16" s="8">
-        <v>12774.19</v>
-      </c>
-      <c r="R16" s="19">
-        <v>153.87881010000001</v>
-      </c>
-      <c r="S16" s="24">
-        <v>180.34</v>
-      </c>
+      <c r="Q16" s="21"/>
+      <c r="R16" s="21"/>
+      <c r="S16" s="21"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A17" s="22">
+      <c r="A17" s="10">
         <v>45748</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="11">
         <v>515</v>
       </c>
       <c r="C17" s="2">
@@ -1693,36 +1572,30 @@
       <c r="K17" s="8">
         <v>13841.67</v>
       </c>
-      <c r="L17" s="14">
+      <c r="L17" s="16">
         <v>180.7</v>
       </c>
-      <c r="M17" s="23">
+      <c r="M17" s="16">
         <v>191.17</v>
       </c>
       <c r="N17" s="8">
         <v>13841.67</v>
       </c>
-      <c r="O17" s="14">
+      <c r="O17" s="16">
         <v>180.7</v>
       </c>
-      <c r="P17" s="23">
+      <c r="P17" s="16">
         <v>191.17</v>
       </c>
-      <c r="Q17" s="8">
-        <v>13501.67</v>
-      </c>
-      <c r="R17" s="19">
-        <v>163.81</v>
-      </c>
-      <c r="S17" s="24">
-        <v>175.58</v>
-      </c>
+      <c r="Q17" s="21"/>
+      <c r="R17" s="21"/>
+      <c r="S17" s="21"/>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A18" s="22">
+      <c r="A18" s="10">
         <v>45778</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="11">
         <v>515</v>
       </c>
       <c r="C18" s="2">
@@ -1756,36 +1629,30 @@
       <c r="K18" s="8">
         <v>13551.61</v>
       </c>
-      <c r="L18" s="14">
+      <c r="L18" s="16">
         <v>205.05</v>
       </c>
-      <c r="M18" s="23">
+      <c r="M18" s="16">
         <v>185.32</v>
       </c>
       <c r="N18" s="8">
         <v>13551.61</v>
       </c>
-      <c r="O18" s="14">
+      <c r="O18" s="16">
         <v>205.05</v>
       </c>
-      <c r="P18" s="23">
+      <c r="P18" s="16">
         <v>175.68</v>
       </c>
-      <c r="Q18" s="8">
-        <v>13400</v>
-      </c>
-      <c r="R18" s="19">
-        <v>197.41</v>
-      </c>
-      <c r="S18" s="24">
-        <v>200.46</v>
-      </c>
+      <c r="Q18" s="21"/>
+      <c r="R18" s="21"/>
+      <c r="S18" s="21"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A19" s="22">
+      <c r="A19" s="10">
         <v>45809</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="11">
         <v>510</v>
       </c>
       <c r="C19" s="2">
@@ -1819,36 +1686,30 @@
       <c r="K19" s="8">
         <v>13710</v>
       </c>
-      <c r="L19" s="14">
+      <c r="L19" s="16">
         <v>238.21</v>
       </c>
-      <c r="M19" s="23">
+      <c r="M19" s="16">
         <v>187.83</v>
       </c>
       <c r="N19" s="8">
         <v>13710</v>
       </c>
-      <c r="O19" s="14">
+      <c r="O19" s="16">
         <v>238.21</v>
       </c>
-      <c r="P19" s="23">
+      <c r="P19" s="16">
         <v>155.66999999999999</v>
       </c>
-      <c r="Q19" s="8">
-        <v>13435</v>
-      </c>
-      <c r="R19" s="19">
-        <v>224.29</v>
-      </c>
-      <c r="S19" s="24">
-        <v>203.15</v>
-      </c>
+      <c r="Q19" s="21"/>
+      <c r="R19" s="21"/>
+      <c r="S19" s="21"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A20" s="22">
+      <c r="A20" s="10">
         <v>45839</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="11">
         <v>510</v>
       </c>
       <c r="C20" s="2">
@@ -1882,36 +1743,30 @@
       <c r="K20" s="8">
         <v>14080.65</v>
       </c>
-      <c r="L20" s="14">
+      <c r="L20" s="16">
         <v>295.68</v>
       </c>
-      <c r="M20" s="23">
+      <c r="M20" s="16">
         <v>206.61</v>
       </c>
       <c r="N20" s="8">
         <v>14080.65</v>
       </c>
-      <c r="O20" s="14">
+      <c r="O20" s="16">
         <v>295.68</v>
       </c>
-      <c r="P20" s="23">
+      <c r="P20" s="16">
         <v>201.61</v>
       </c>
-      <c r="Q20" s="8">
-        <v>13635.48</v>
-      </c>
-      <c r="R20" s="19">
-        <v>272.77</v>
-      </c>
-      <c r="S20" s="24">
-        <v>290.02</v>
-      </c>
+      <c r="Q20" s="21"/>
+      <c r="R20" s="21"/>
+      <c r="S20" s="21"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A21" s="22">
+      <c r="A21" s="10">
         <v>45870</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="11">
         <v>510</v>
       </c>
       <c r="C21" s="2">
@@ -1945,36 +1800,30 @@
       <c r="K21" s="8">
         <v>14325.81</v>
       </c>
-      <c r="L21" s="14">
+      <c r="L21" s="16">
         <v>334.32</v>
       </c>
-      <c r="M21" s="23">
+      <c r="M21" s="16">
         <v>223.94</v>
       </c>
       <c r="N21" s="8">
         <v>14325.81</v>
       </c>
-      <c r="O21" s="14">
+      <c r="O21" s="16">
         <v>334.32</v>
       </c>
-      <c r="P21" s="23">
+      <c r="P21" s="16">
         <v>218.94</v>
       </c>
-      <c r="Q21" s="8">
-        <v>13990.32</v>
-      </c>
-      <c r="R21" s="19">
-        <v>316.76</v>
-      </c>
-      <c r="S21" s="24">
-        <v>270.11</v>
-      </c>
+      <c r="Q21" s="21"/>
+      <c r="R21" s="21"/>
+      <c r="S21" s="21"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A22" s="22">
+      <c r="A22" s="10">
         <v>45901</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="11">
         <v>510</v>
       </c>
       <c r="C22" s="2">
@@ -2008,36 +1857,30 @@
       <c r="K22" s="8">
         <v>13150</v>
       </c>
-      <c r="L22" s="14">
+      <c r="L22" s="16">
         <v>241.2</v>
       </c>
-      <c r="M22" s="23">
+      <c r="M22" s="16">
         <v>202</v>
       </c>
       <c r="N22" s="8">
         <v>13150</v>
       </c>
-      <c r="O22" s="14">
+      <c r="O22" s="16">
         <v>241.2</v>
       </c>
-      <c r="P22" s="23">
+      <c r="P22" s="16">
         <v>197</v>
       </c>
-      <c r="Q22" s="8">
-        <v>12566.67</v>
-      </c>
-      <c r="R22" s="19">
-        <v>211.24</v>
-      </c>
-      <c r="S22" s="24">
-        <v>186.85</v>
-      </c>
+      <c r="Q22" s="21"/>
+      <c r="R22" s="21"/>
+      <c r="S22" s="21"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A23" s="20">
+      <c r="A23" s="14">
         <v>45931</v>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="11">
         <v>510</v>
       </c>
       <c r="C23" s="2">
@@ -2071,36 +1914,34 @@
       <c r="K23" s="8">
         <v>11632</v>
       </c>
-      <c r="L23" s="17">
+      <c r="L23" s="19">
         <v>188.49</v>
       </c>
-      <c r="M23" s="23">
+      <c r="M23" s="16">
         <v>190.42</v>
       </c>
       <c r="N23" s="8">
         <v>11630</v>
       </c>
-      <c r="O23" s="14">
+      <c r="O23" s="16">
         <v>188.49</v>
       </c>
-      <c r="P23" s="23">
+      <c r="P23" s="16">
         <v>185.42</v>
       </c>
-      <c r="Q23" s="8">
-        <v>11641.94</v>
-      </c>
-      <c r="R23" s="19">
+      <c r="Q23" s="21"/>
+      <c r="R23" s="21">
         <v>240.9</v>
       </c>
-      <c r="S23" s="24">
+      <c r="S23" s="21">
         <v>172.48</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A24" s="20">
+      <c r="A24" s="14">
         <v>45962</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="11">
         <v>510</v>
       </c>
       <c r="C24" s="2">
@@ -2134,36 +1975,34 @@
       <c r="K24" s="8">
         <v>11767.383669999999</v>
       </c>
-      <c r="L24" s="17">
+      <c r="L24" s="19">
         <v>175.89</v>
       </c>
-      <c r="M24" s="23">
+      <c r="M24" s="16">
         <v>197.73</v>
       </c>
       <c r="N24" s="8">
         <v>11768.821669999999</v>
       </c>
-      <c r="O24" s="17">
+      <c r="O24" s="19">
         <v>175.89</v>
       </c>
-      <c r="P24" s="23">
+      <c r="P24" s="16">
         <v>192.73</v>
       </c>
-      <c r="Q24" s="8">
-        <v>11743.33</v>
-      </c>
-      <c r="R24" s="19">
+      <c r="Q24" s="21"/>
+      <c r="R24" s="21">
         <v>242.3</v>
       </c>
-      <c r="S24" s="24">
+      <c r="S24" s="21">
         <v>170.54</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A25" s="20">
+      <c r="A25" s="14">
         <v>45992</v>
       </c>
-      <c r="B25" s="10">
+      <c r="B25" s="11">
         <v>510</v>
       </c>
       <c r="C25" s="2">
@@ -2196,36 +2035,34 @@
       <c r="K25" s="8">
         <v>11983.51</v>
       </c>
-      <c r="L25" s="17">
+      <c r="L25" s="19">
         <v>165.07</v>
       </c>
-      <c r="M25" s="23">
+      <c r="M25" s="16">
         <v>203.23</v>
       </c>
       <c r="N25" s="8">
         <v>11984.84</v>
       </c>
-      <c r="O25" s="14">
+      <c r="O25" s="16">
         <v>203.23</v>
       </c>
-      <c r="P25" s="23">
+      <c r="P25" s="16">
         <v>198.23</v>
       </c>
-      <c r="Q25" s="8">
-        <v>11830.65</v>
-      </c>
-      <c r="R25" s="19">
+      <c r="Q25" s="21"/>
+      <c r="R25" s="21">
         <v>240.98</v>
       </c>
-      <c r="S25" s="24">
+      <c r="S25" s="21">
         <v>159.74</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A26" s="20">
+      <c r="A26" s="14">
         <v>46048</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="11">
         <v>510</v>
       </c>
       <c r="C26" s="2">
@@ -2239,322 +2076,158 @@
         <v>1669000</v>
       </c>
       <c r="F26" s="6">
-        <v>1203000</v>
+        <v>1110000</v>
       </c>
       <c r="G26" s="6">
         <f>E26+F26</f>
-        <v>2872000</v>
+        <v>2779000</v>
       </c>
       <c r="H26" s="6">
-        <v>1327000</v>
+        <v>1000000</v>
       </c>
       <c r="I26" s="6">
         <f t="shared" si="4"/>
-        <v>1545000</v>
-      </c>
-      <c r="J26" s="16">
+        <v>1779000</v>
+      </c>
+      <c r="J26" s="18">
         <f>I26/H26</f>
-        <v>1.1642803315749812</v>
-      </c>
-      <c r="K26" s="8">
-        <v>12120</v>
-      </c>
-      <c r="L26" s="11">
-        <v>191.85</v>
-      </c>
-      <c r="M26" s="2">
-        <v>203.71</v>
-      </c>
-      <c r="N26" s="8">
-        <v>12120</v>
-      </c>
-      <c r="O26" s="13">
-        <v>191.85</v>
-      </c>
-      <c r="P26" s="2">
-        <v>206.16</v>
-      </c>
-      <c r="Q26" s="8">
-        <v>11925</v>
-      </c>
-      <c r="R26" s="19">
-        <v>239.16</v>
-      </c>
-      <c r="S26" s="24">
-        <v>184.25</v>
-      </c>
+        <v>1.7789999999999999</v>
+      </c>
+      <c r="K26" s="8"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="8"/>
+      <c r="O26" s="15"/>
+      <c r="P26" s="12"/>
+      <c r="Q26" s="21"/>
+      <c r="R26" s="21"/>
+      <c r="S26" s="21"/>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A27" s="20">
-        <v>46079</v>
-      </c>
-      <c r="B27" s="10">
-        <v>510</v>
-      </c>
-      <c r="C27" s="2">
-        <v>434.46</v>
-      </c>
-      <c r="D27" s="2">
-        <v>47.148400000000002</v>
-      </c>
-      <c r="E27" s="6">
-        <f>I26</f>
-        <v>1545000</v>
-      </c>
-      <c r="F27" s="6">
-        <v>355000</v>
-      </c>
-      <c r="G27" s="6">
-        <f>E27+F27</f>
-        <v>1900000</v>
-      </c>
-      <c r="H27" s="6">
-        <v>750000</v>
-      </c>
-      <c r="I27" s="6">
-        <f t="shared" si="4"/>
-        <v>1150000</v>
-      </c>
-      <c r="J27" s="16">
-        <f>I27/H27</f>
-        <v>1.5333333333333334</v>
-      </c>
-      <c r="K27" s="8">
-        <v>12430</v>
-      </c>
-      <c r="L27" s="11">
-        <v>202.84</v>
-      </c>
-      <c r="M27" s="2">
-        <v>213.93</v>
-      </c>
-      <c r="N27" s="8">
-        <v>12430</v>
-      </c>
-      <c r="O27" s="13">
-        <v>202.84</v>
-      </c>
-      <c r="P27" s="2">
-        <v>214.36</v>
-      </c>
-      <c r="Q27" s="8">
-        <v>11896</v>
-      </c>
-      <c r="R27" s="19">
-        <v>239.35</v>
-      </c>
-      <c r="S27" s="24">
-        <v>184.25</v>
-      </c>
+      <c r="A27" s="12"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="8"/>
+      <c r="O27" s="15"/>
+      <c r="P27" s="12"/>
+      <c r="Q27" s="21"/>
+      <c r="R27" s="21"/>
+      <c r="S27" s="21"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A28" s="20">
-        <v>46107</v>
-      </c>
-      <c r="B28" s="10">
-        <v>510</v>
-      </c>
-      <c r="C28" s="2">
-        <v>434.46</v>
-      </c>
-      <c r="D28" s="2">
-        <v>50</v>
-      </c>
-      <c r="E28" s="6">
-        <f>I27</f>
-        <v>1150000</v>
-      </c>
-      <c r="F28" s="6">
-        <v>826000</v>
-      </c>
-      <c r="G28" s="6">
-        <f>E28+F28</f>
-        <v>1976000</v>
-      </c>
-      <c r="H28" s="6">
-        <v>1093000</v>
-      </c>
-      <c r="I28" s="6">
-        <f t="shared" ref="I28:I30" si="9">G28-H28</f>
-        <v>883000</v>
-      </c>
-      <c r="J28" s="16">
-        <f>I28/H28</f>
-        <v>0.80786825251601102</v>
-      </c>
-      <c r="K28" s="8">
-        <v>14268</v>
-      </c>
-      <c r="L28" s="11">
-        <v>212.58</v>
-      </c>
-      <c r="M28" s="2">
-        <v>215.1</v>
-      </c>
-      <c r="N28" s="8">
-        <v>14268</v>
-      </c>
-      <c r="O28" s="11">
-        <v>212.58</v>
-      </c>
-      <c r="P28" s="2">
-        <v>215.1</v>
-      </c>
-      <c r="Q28" s="8">
-        <v>13351.61</v>
-      </c>
-      <c r="R28" s="19">
-        <v>168.35</v>
-      </c>
-      <c r="S28" s="24">
-        <v>244.39</v>
-      </c>
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="12"/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="15"/>
+      <c r="P28" s="12"/>
+      <c r="Q28" s="21"/>
+      <c r="R28" s="21"/>
+      <c r="S28" s="21"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A29" s="30">
-        <v>46138</v>
-      </c>
-      <c r="B29" s="25">
-        <v>515</v>
-      </c>
-      <c r="C29" s="26">
-        <v>461</v>
-      </c>
-      <c r="D29" s="26">
-        <v>53</v>
-      </c>
-      <c r="E29" s="27">
-        <f>I28</f>
-        <v>883000</v>
-      </c>
-      <c r="F29" s="28">
-        <v>1634000</v>
-      </c>
-      <c r="G29" s="27">
-        <f>E29+F29</f>
-        <v>2517000</v>
-      </c>
-      <c r="H29" s="28">
-        <v>1044000</v>
-      </c>
-      <c r="I29" s="27">
-        <f t="shared" si="9"/>
-        <v>1473000</v>
-      </c>
-      <c r="J29" s="29">
-        <f>I29/H29</f>
-        <v>1.4109195402298851</v>
-      </c>
-      <c r="K29" s="8">
-        <v>14600</v>
-      </c>
-      <c r="L29" s="11">
-        <v>222</v>
-      </c>
-      <c r="M29" s="2">
-        <v>247</v>
-      </c>
-      <c r="N29" s="8">
-        <v>14600</v>
-      </c>
-      <c r="O29" s="13">
-        <v>222</v>
-      </c>
-      <c r="P29" s="2">
-        <v>247</v>
-      </c>
-      <c r="Q29" s="8">
-        <v>14000</v>
-      </c>
-      <c r="R29" s="31">
-        <v>176.13</v>
-      </c>
-      <c r="S29" s="24">
-        <v>190</v>
-      </c>
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="12"/>
+      <c r="N29" s="8"/>
+      <c r="O29" s="15"/>
+      <c r="P29" s="12"/>
+      <c r="Q29" s="21"/>
+      <c r="R29" s="21"/>
+      <c r="S29" s="21"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A30" s="30">
-        <v>46168</v>
-      </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="26">
-        <v>52</v>
-      </c>
-      <c r="E30" s="6">
-        <f>I29</f>
-        <v>1473000</v>
-      </c>
-      <c r="F30" s="11">
-        <v>1000000</v>
-      </c>
-      <c r="G30" s="11">
-        <f>E30+F30</f>
-        <v>2473000</v>
-      </c>
-      <c r="H30" s="11">
-        <v>1000000</v>
-      </c>
-      <c r="I30" s="11">
-        <f t="shared" si="9"/>
-        <v>1473000</v>
-      </c>
-      <c r="J30" s="11">
-        <f>I30/H30</f>
-        <v>1.4730000000000001</v>
-      </c>
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
       <c r="K30" s="8"/>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11"/>
+      <c r="L30" s="12"/>
+      <c r="M30" s="12"/>
       <c r="N30" s="8"/>
-      <c r="O30" s="13"/>
-      <c r="P30" s="11"/>
-      <c r="Q30" s="19"/>
-      <c r="R30" s="19"/>
-      <c r="S30" s="19"/>
+      <c r="O30" s="15"/>
+      <c r="P30" s="12"/>
+      <c r="Q30" s="21"/>
+      <c r="R30" s="21"/>
+      <c r="S30" s="21"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A31" s="11"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="11"/>
-      <c r="J31" s="11"/>
+      <c r="A31" s="12"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
       <c r="K31" s="8"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
+      <c r="L31" s="12"/>
+      <c r="M31" s="12"/>
       <c r="N31" s="8"/>
-      <c r="O31" s="13"/>
-      <c r="P31" s="11"/>
-      <c r="Q31" s="19"/>
-      <c r="R31" s="19"/>
-      <c r="S31" s="19"/>
+      <c r="O31" s="15"/>
+      <c r="P31" s="12"/>
+      <c r="Q31" s="21"/>
+      <c r="R31" s="21"/>
+      <c r="S31" s="21"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A32" s="11"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="11"/>
+      <c r="A32" s="12"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
       <c r="K32" s="8"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
+      <c r="L32" s="12"/>
+      <c r="M32" s="12"/>
       <c r="N32" s="8"/>
-      <c r="O32" s="13"/>
-      <c r="P32" s="11"/>
-      <c r="Q32" s="19"/>
-      <c r="R32" s="19"/>
-      <c r="S32" s="19"/>
+      <c r="O32" s="15"/>
+      <c r="P32" s="12"/>
+      <c r="Q32" s="21"/>
+      <c r="R32" s="21"/>
+      <c r="S32" s="21"/>
     </row>
     <row r="33" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O33" s="1"/>

</xml_diff>